<commit_message>
Initial commit - Cham cong Ngay phep Dao tao Ngoai gio Ho so ..
</commit_message>
<xml_diff>
--- a/thong_tin_nguoi_lao_dong_tao_user.xlsx
+++ b/thong_tin_nguoi_lao_dong_tao_user.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lequocvan/Downloads/Cham_cong_Ngoai_gio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5ADA8A0-5AD8-1E44-B51C-67AFD9BCC70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4053199F-DA5C-2043-B96B-0E59E9B11DC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="460" windowWidth="25220" windowHeight="10240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>id</t>
   </si>
@@ -79,59 +79,16 @@
   </si>
   <si>
     <t>created_at</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Trưởng phòng</t>
-  </si>
-  <si>
-    <t>Phan Thùy Dương</t>
-  </si>
-  <si>
-    <t>Nữ</t>
-  </si>
-  <si>
-    <t>0915652222</t>
-  </si>
-  <si>
-    <t>duongphanthuy1@agribank.com.vn</t>
-  </si>
-  <si>
-    <t>200713234</t>
-  </si>
-  <si>
-    <t>PCRT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-  </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -142,7 +99,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -150,60 +107,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -516,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
@@ -587,57 +499,10 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="18" x14ac:dyDescent="0.2">
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="1">
-        <v>29514</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="2">
-        <v>43466</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" t="s">
-        <v>18</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2" s="3">
-        <v>46245.339699074073</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="G3" s="4"/>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="G2" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" xr:uid="{D6CA01CC-2DBA-B640-9C36-3E686C5EAAD7}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>